<commit_message>
Wiki avions : V3 (textes FR, rôles, noms d'emplacements) et V4 (aircraft.json, mise à jour sans recompiler)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ta6XHrP5piK3ygC9quASBg
</commit_message>
<xml_diff>
--- a/data/Avions_wiki.xlsx
+++ b/data/Avions_wiki.xlsx
@@ -993,7 +993,11 @@
         </is>
       </c>
       <c r="F2" s="4" t="n"/>
-      <c r="G2" s="4" t="n"/>
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>Des MiG-15 en plein '85 :wilt: :sob:</t>
+        </is>
+      </c>
       <c r="H2" s="4" t="n"/>
       <c r="I2" t="inlineStr">
         <is>
@@ -1153,8 +1157,16 @@
           <t>Avion à hélice (turbopropulseur)</t>
         </is>
       </c>
-      <c r="F3" s="4" t="n"/>
-      <c r="G3" s="4" t="n"/>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>Contre-insurrection · Appui aérien rapproché</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>Conçu pour la contre-insurrection et les conflits de faible intensité, le CI-22 Cricket dispose d'un train d'atterrissage robuste et de capacités de décollage et d'atterrissage courts, qui lui permettent d'opérer depuis des terrains non préparés. S'il manque de vitesse et de capacité de survie, le CI-22 offre une agilité remarquable et peut emporter un large éventail d'armes.</t>
+        </is>
+      </c>
       <c r="H3" s="4" t="n"/>
       <c r="I3" t="inlineStr">
         <is>
@@ -1317,8 +1329,16 @@
           <t>Avion à hélice (turbopropulseur)</t>
         </is>
       </c>
-      <c r="F4" s="4" t="n"/>
-      <c r="G4" s="4" t="n"/>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Contre-insurrection · Attaque au sol · Entraînement</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>Le Hartnell-Wesley OA-27 Cavalier est un avion léger d'entraînement, d'attaque et de contre-insurrection en service dans l'État primévien et la PALAAF. Conçu avant la révolution dans l'un des micro-États primévien, le Cavalier est l'appareil de choix pour les opérations d'attaque de faible intensité, les escarmouches frontalières et la formation intermédiaire des pilotes. Il est fiable, robuste et remarquablement peu coûteux à acquérir et à entretenir.</t>
+        </is>
+      </c>
       <c r="H4" s="4" t="n"/>
       <c r="I4" t="inlineStr">
         <is>
@@ -1477,8 +1497,16 @@
           <t>Hélicoptère</t>
         </is>
       </c>
-      <c r="F5" s="4" t="n"/>
-      <c r="G5" s="4" t="n"/>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Reconnaissance · Hélicoptère d'attaque</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>Le RAH-72 est un hélicoptère de reconnaissance et d'attaque légère. Capable d'emporter un bon nombre de munitions légères, c'est un monoplace biturbine à rotors coaxiaux et empennage en V, avec des soutes internes sous le fuselage et quatre pylônes externes sur des ailettes dont les extrémités portent ses lance-leurres. Il bénéficie d'une mise en forme à facettes peu observable, d'excellents capteurs optiques et d'un grand radar de triangulation au sol monté au sommet du mât rotor, qui détecte unités terrestres et navires à longue distance.</t>
+        </is>
+      </c>
       <c r="H5" s="4" t="n"/>
       <c r="I5" t="inlineStr">
         <is>
@@ -1628,8 +1656,16 @@
           <t>Avion à réaction</t>
         </is>
       </c>
-      <c r="F6" s="4" t="n"/>
-      <c r="G6" s="4" t="n"/>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>Entraînement · Attaque au sol</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>Avion d'entraînement avancé à réaction, bien adapté aux missions de combat léger, le T/A-30 est très manœuvrant à basse et moyenne vitesse et pardonne les erreurs de pilotage. Particulièrement à l'aise dans les frappes à basse altitude, le Compass dispose de gouvernes redondantes et de deux réacteurs qui améliorent sa capacité de survie.</t>
+        </is>
+      </c>
       <c r="H6" s="4" t="n"/>
       <c r="I6" t="inlineStr">
         <is>
@@ -1792,8 +1828,16 @@
           <t>Avion à décollage vertical (jets)</t>
         </is>
       </c>
-      <c r="F7" s="4" t="n"/>
-      <c r="G7" s="4" t="n"/>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Entraînement · Attaque au sol · Embarqué (porte-avions)</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>Doté d'un système unique de poussée canalisée à trois tuyères, cet avion d'entraînement sert aussi d'avion d'attaque économique à décollage vertical. Le Vagrant est très manœuvrant et atteint des vitesses transsoniques ; il dispose aussi d'un radar qui lui permet d'engager des cibles aériennes au-delà de la portée visuelle. Bien qu'il n'ait pas de furtivité avancée, le VT-7 reste la colonne vertébrale de l'aéronavale de la BDF.</t>
+        </is>
+      </c>
       <c r="H7" s="4" t="n"/>
       <c r="I7" t="inlineStr">
         <is>
@@ -1959,8 +2003,16 @@
           <t>Hélicoptère</t>
         </is>
       </c>
-      <c r="F8" s="4" t="n"/>
-      <c r="G8" s="4" t="n"/>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>Hélicoptère utilitaire · Transport</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>Conçu pour un programme PALA de transport vertical rapide dans les années 2050, l'UH-90 a été pensé comme un hélicoptère utilitaire combiné de taille moyenne, mais il a depuis reçu de nombreux points d'emport qui lui permettent de servir d'appareil d'appui feu. Doté d'un rotor rigide coaxial et de deux soufflantes carénées turbo-électriques réversibles en configuration propulsive, l'Ibis atteint rapidement de hautes vitesses de croisière avant de décélérer jusqu'à un atterrissage vertical en moins de 30 secondes.</t>
+        </is>
+      </c>
       <c r="H8" s="4" t="n"/>
       <c r="I8" t="inlineStr">
         <is>
@@ -2114,8 +2166,16 @@
           <t>Hélicoptère</t>
         </is>
       </c>
-      <c r="F9" s="4" t="n"/>
-      <c r="G9" s="4" t="n"/>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Hélicoptère d'attaque</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>Le SAH-46 Chicane conserve la configuration classique d'un hélicoptère d'attaque tout en intégrant des améliorations qui en font toujours une présence redoutable sur le champ de bataille de la fin du XXIe siècle. Sa technologie furtive de pointe lui permet de lancer des attaques surprises depuis l'abri du relief, puis de disparaître des radars sans laisser de trace.</t>
+        </is>
+      </c>
       <c r="H9" s="4" t="n"/>
       <c r="I9" t="inlineStr">
         <is>
@@ -2272,8 +2332,16 @@
           <t>Avion à réaction</t>
         </is>
       </c>
-      <c r="F10" s="4" t="n"/>
-      <c r="G10" s="4" t="n"/>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>Supériorité aérienne · Chasseur</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>Malgré une conception ancienne, ce chasseur léger supersonique est exceptionnellement agile et très adapté aux missions de supériorité aérienne, avec des options d'attaque au sol limitées à basse altitude. Ses deux réacteurs lui donnent un rapport poussée/poids et une vitesse de pointe incroyables, tandis qu'une soute interne axiale réduit la traînée de la charge.</t>
+        </is>
+      </c>
       <c r="H10" s="4" t="n"/>
       <c r="I10" t="inlineStr">
         <is>
@@ -2439,8 +2507,16 @@
           <t>Avion à hélice (turbopropulseur)</t>
         </is>
       </c>
-      <c r="F11" s="4" t="n"/>
-      <c r="G11" s="4" t="n"/>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Appui aérien rapproché · Attaque au sol · Lutte antinavire</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>Le Brawler est une plateforme fiable et robuste, conçue pour emporter de grandes quantités d'armes de précision. Ses propfans de pointe allient endurance et vitesse respectable, tandis que ses gouvernes redondantes, ses moteurs isolés et le lourd blindage de son cockpit lui assurent une excellente capacité de survie. L'A-19 est dans son élément face aux convois de véhicules, aux défenses antiaériennes courte portée dispersées ou aux navires opérant en eaux côtières.</t>
+        </is>
+      </c>
       <c r="H11" s="4" t="n"/>
       <c r="I11" t="inlineStr">
         <is>
@@ -2606,8 +2682,16 @@
           <t>Convertible à rotors basculants</t>
         </is>
       </c>
-      <c r="F12" s="4" t="n"/>
-      <c r="G12" s="4" t="n"/>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>Alliant capacité de levage vertical et 20 tonnes de capacité d'emport, ce grand quadrimoteur à ailes basculantes peut livrer des approvisionnements vitaux aux positions avancées ou servir d'appareil d'appui feu polyvalent. Ses 4 rotors sont reliés par des arbres de transmission internes, ce qui permet au Tarantula de continuer à voler après avoir encaissé des dégâts importants.</t>
+        </is>
+      </c>
       <c r="H12" s="4" t="n"/>
       <c r="I12" t="inlineStr">
         <is>
@@ -2759,7 +2843,11 @@
         </is>
       </c>
       <c r="F13" s="4" t="n"/>
-      <c r="G13" s="4" t="n"/>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>Bien que plus que centenaire, le F-16 reste un pilier des forces aériennes du monde entier, ses dernières variantes Block 165 étant en service aussi bien dans la BDAF que dans la PALAAF. Les programmes de modernisation et un lobbying acharné l'ont maintenu dans la course : le Viper est vraiment éternel.</t>
+        </is>
+      </c>
       <c r="H13" s="4" t="n"/>
       <c r="I13" t="inlineStr">
         <is>
@@ -2930,8 +3018,16 @@
           <t>Avion à réaction</t>
         </is>
       </c>
-      <c r="F14" s="4" t="n"/>
-      <c r="G14" s="4" t="n"/>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>Chasseur</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>Une conception plus ancienne mais éprouvée, qui remonte à la révolution primévienne. L'Agni est un chasseur monoréacteur tout temps doté d'un grand nombre de points d'emport pour plus de souplesse. Sans aucune soute interne, l'appareil est plus facile à détecter que les modèles plus modernes.</t>
+        </is>
+      </c>
       <c r="H14" s="4" t="n"/>
       <c r="I14" t="inlineStr">
         <is>
@@ -3102,8 +3198,16 @@
           <t>Avion à réaction</t>
         </is>
       </c>
-      <c r="F15" s="4" t="n"/>
-      <c r="G15" s="4" t="n"/>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>Supériorité aérienne</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>Le FS-12 Revoker est conçu avant tout pour l'agilité : il est capable de manœuvres extrêmes à presque toutes les vitesses. Ses soutes internes réduisent la traînée et lui permettent d'atteindre des vitesses supersoniques même à basse altitude et lourdement armé. Moins furtif que les chasseurs plus récents, le Revoker reste un moyen économique d'obtenir la supériorité aérienne.</t>
+        </is>
+      </c>
       <c r="H15" s="4" t="n"/>
       <c r="I15" t="inlineStr">
         <is>
@@ -3269,8 +3373,16 @@
           <t>Avion à réaction</t>
         </is>
       </c>
-      <c r="F16" s="4" t="n"/>
-      <c r="G16" s="4" t="n"/>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>Multirôle · Embarqué (porte-avions)</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>Chasseur multirôle compact et avancé, le Vortex peut opérer à la verticale depuis de petits porte-avions et rester indétecté grâce à une furtivité exceptionnelle. Rapide, agile et furtif quand il est peu chargé, il perd une partie de ces qualités sous une lourde charge d'armement.</t>
+        </is>
+      </c>
       <c r="H16" s="4" t="n"/>
       <c r="I16" t="inlineStr">
         <is>
@@ -3436,8 +3548,16 @@
           <t>Avion à réaction</t>
         </is>
       </c>
-      <c r="F17" s="4" t="n"/>
-      <c r="G17" s="4" t="n"/>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>Frappe furtive</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>Avion de frappe subsonique rapide à très faible observabilité, doté de deux réacteurs F404 sans postcombustion, de commandes de vol électriques numériques, d'un système de désignation électro-optique et de deux soutes internes. Un large choix de chargements de bombes et de missiles compatibles offre un jeu varié. Soutes fermées, les armes internes restent masquées au radar ; ouvrir une soute ou sortir le train augmente la signature radar. Un brouilleur radar actif fixe est installé dans chaque chargement : sélectionne-le comme arme, désigne une cible radar suivie et maintiens le tir pour brouiller. Maintenir le frein de roues pendant un roulage d'atterrissage valide déploie le parachute de freinage (à usage unique) une fois les trois roues au sol et l'appareil aligné sur sa trajectoire.</t>
+        </is>
+      </c>
       <c r="H17" s="4" t="n"/>
       <c r="I17" t="inlineStr">
         <is>
@@ -3608,8 +3728,16 @@
           <t>Avion à réaction</t>
         </is>
       </c>
-      <c r="F18" s="4" t="n"/>
-      <c r="G18" s="4" t="n"/>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>Multirôle · Embarqué (porte-avions)</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>Grand chasseur multirôle biréacteur apte à l'embarquement, l'Ifrit convient aussi bien à la supériorité aérienne qu'à l'attaque au sol. Il offre une poussée et une maniabilité excellentes, une signature radar réduite et des capteurs puissants. Deux soutes internes, plus deux soutes latérales pour missiles à guidage infrarouge, permettent à l'Ifrit d'emporter une charge interne importante sans nuire à sa furtivité ni à sa vitesse de pointe.</t>
+        </is>
+      </c>
       <c r="H18" s="4" t="n"/>
       <c r="I18" t="inlineStr">
         <is>
@@ -3775,8 +3903,16 @@
           <t>Avion à réaction</t>
         </is>
       </c>
-      <c r="F19" s="4" t="n"/>
-      <c r="G19" s="4" t="n"/>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>Multirôle</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>Conçu au tournant du siècle, le FS-3 Ternion est un grand chasseur multirôle biréacteur. D'abord développé pour de longues patrouilles au-dessus du Pacifique, il a ensuite été adapté à des besoins opérationnels croissants. Malgré l'absence de furtivité, des modernisations régulières ont permis au Ternion de rester un défenseur fiable du Heartland.</t>
+        </is>
+      </c>
       <c r="H19" s="4" t="n"/>
       <c r="I19" t="inlineStr">
         <is>
@@ -3947,8 +4083,16 @@
           <t>Avion à réaction</t>
         </is>
       </c>
-      <c r="F20" s="4" t="n"/>
-      <c r="G20" s="4" t="n"/>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>Guerre électronique · SEAD</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>L'EW-25 est un avion de soutien à décollage court et atterrissage vertical (STOVL) doté de puissants systèmes de guerre électronique. Capable de trianguler la position des radars, de brouiller les installations radar ennemies, de neutraliser les défenses antiaériennes et même d'abattre des missiles avec un laser à haute énergie, un seul Medusa peut facilement renverser le cours d'une bataille.</t>
+        </is>
+      </c>
       <c r="H20" s="4" t="n"/>
       <c r="I20" t="inlineStr">
         <is>
@@ -4111,8 +4255,16 @@
           <t>Avion à réaction</t>
         </is>
       </c>
-      <c r="F21" s="4" t="n"/>
-      <c r="G21" s="4" t="n"/>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>Transport · Bombardier</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>Plus gros appareil d'Aryx Dynamics à ce jour, le MC-260 Chimera est un avion cargo lourd polyvalent, conçu pour des opérations multirôles lourdes et rustiques dans des conditions spartiates, près des lignes de front. Il offre des performances de décollage et d'atterrissage courts à faible charge grâce à son aile soufflée et à ses inverseurs de poussée, et tient dans les hangars moyens existants grâce à son gouvernail à volets divisés et à ses dérives ventrales uniques. Le Chimera peut servir de canonnière, de bombardier, d'avion de guet aérien (AEW) et de transport de fret.</t>
+        </is>
+      </c>
       <c r="H21" s="4" t="n"/>
       <c r="I21" t="inlineStr">
         <is>
@@ -4278,8 +4430,16 @@
           <t>Avion à réaction</t>
         </is>
       </c>
-      <c r="F22" s="4" t="n"/>
-      <c r="G22" s="4" t="n"/>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>Supériorité aérienne · Attaque au sol</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>Proposé à la fin des années 2040, en pleine Troisième Guerre mondiale, comme programme de modernisation et de refonte du F-22C d'exportation, le F-22E Strike Raptor reprend la forme bien connue du F-22 en y ajoutant une paire d'EOTS intégrés aux arêtes du fuselage central pour guider les munitions de précision, ainsi qu'une soute agrandie et approfondie pour emporter de gros volumes d'armement. Excellente agilité, poussée vectorielle, nacelles d'armes furtives possibles sur ses pylônes d'aile intérieurs, et désormais tout à fait capable d'attaque au sol comme de domination aérienne : le F-22E est aussi féroce que l'était son modèle original un demi-siècle plus tôt.</t>
+        </is>
+      </c>
       <c r="H22" s="4" t="n"/>
       <c r="I22" t="inlineStr">
         <is>
@@ -4441,8 +4601,16 @@
           <t>Avion à réaction</t>
         </is>
       </c>
-      <c r="F23" s="4" t="n"/>
-      <c r="G23" s="4" t="n"/>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>Bombardier furtif</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>Avec ses moteurs puissants, sa silhouette furtive et ses 4 grandes soutes internes, le SFB-81 Darkreach est un bombardier redoutable capable de délivrer des armes conventionnelles comme nucléaires. Son aile volante intégrée lui permet d'opérer dans des régimes de vol variés, de la pénétration à très basse altitude au bombardement stratégique à distance de sécurité.</t>
+        </is>
+      </c>
       <c r="H23" s="4" t="n"/>
       <c r="I23" t="inlineStr">
         <is>
@@ -4605,8 +4773,16 @@
           <t>Avion à réaction à ailes à géométrie variable</t>
         </is>
       </c>
-      <c r="F24" s="4" t="n"/>
-      <c r="G24" s="4" t="n"/>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>Intercepteur · Embarqué (porte-avions)</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>Le FS-41 Eclipse est un grand intercepteur embarqué biréacteur supersonique, conçu pour localiser, intercepter et détruire les cibles de grande valeur avant qu'elles ne menacent l'espace aérien allié et les groupes aéronavals. Il allie des vitesses supérieures à Mach 2, un radar extraordinairement puissant et une furtivité impressionnante pour son rôle d'interception et de domination, renforcés par son armement emblématique, le missile AAM-45 Sabre. Ses ailes à géométrie variable le rendent en outre très agile, et il peut emporter une charge air-sol limitée pour des missions variées.</t>
+        </is>
+      </c>
       <c r="H24" s="4" t="n"/>
       <c r="I24" t="inlineStr">
         <is>
@@ -4777,8 +4953,16 @@
           <t>Avion à réaction à ailes à géométrie variable</t>
         </is>
       </c>
-      <c r="F25" s="4" t="n"/>
-      <c r="G25" s="4" t="n"/>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>Bombardier · Guerre électronique</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>L'Alkyon AB-4 est un bombardier supersonique avancé doté de capacités de guerre électronique, conçu pour délivrer discrètement des charges nucléaires ou conventionnelles sur des cibles de grande valeur. Ses 4 réacteurs à postcombustion et ses ailes à géométrie variable lui donnent une vitesse de pointe incroyable et assez de maniabilité pour échapper aux menaces aériennes. En cas de dégâts critiques, une capsule d'évacuation permet à l'équipage de s'éjecter en sécurité à toute altitude et à toute vitesse.</t>
+        </is>
+      </c>
       <c r="H25" s="4" t="n"/>
       <c r="I25" t="inlineStr">
         <is>
@@ -5038,7 +5222,11 @@
           <t>Left Internal Cannons</t>
         </is>
       </c>
-      <c r="E2" s="7" t="n"/>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>Canons internes gauches</t>
+        </is>
+      </c>
       <c r="F2" t="inlineStr">
         <is>
           <t>oui</t>
@@ -5085,7 +5273,11 @@
           <t>Right Internal Cannon</t>
         </is>
       </c>
-      <c r="E3" s="7" t="n"/>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>Canon interne droit</t>
+        </is>
+      </c>
       <c r="F3" t="inlineStr">
         <is>
           <t>oui</t>
@@ -5132,7 +5324,11 @@
           <t>Wing Pylons</t>
         </is>
       </c>
-      <c r="E4" s="7" t="n"/>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>Pylônes d'aile</t>
+        </is>
+      </c>
       <c r="F4" t="inlineStr">
         <is>
           <t>oui</t>
@@ -5187,7 +5383,11 @@
           <t>Tail Hook</t>
         </is>
       </c>
-      <c r="E5" s="7" t="n"/>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>Crochet d'appontage</t>
+        </is>
+      </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
           <t>non (sans arme)</t>
@@ -5233,7 +5433,11 @@
           <t>Internal guns</t>
         </is>
       </c>
-      <c r="E6" s="7" t="n"/>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>Canons internes</t>
+        </is>
+      </c>
       <c r="F6" t="inlineStr">
         <is>
           <t>oui</t>
@@ -5288,7 +5492,11 @@
           <t>Ventral Hardpoint</t>
         </is>
       </c>
-      <c r="E7" s="7" t="n"/>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>Point d'emport ventral</t>
+        </is>
+      </c>
       <c r="F7" t="inlineStr">
         <is>
           <t>oui</t>
@@ -5343,7 +5551,11 @@
           <t>Fuselage Pylons</t>
         </is>
       </c>
-      <c r="E8" s="7" t="n"/>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>Pylônes de fuselage</t>
+        </is>
+      </c>
       <c r="F8" t="inlineStr">
         <is>
           <t>oui</t>
@@ -5398,7 +5610,11 @@
           <t>Inner Wing Pylons</t>
         </is>
       </c>
-      <c r="E9" s="7" t="n"/>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>Pylônes d'aile intérieurs</t>
+        </is>
+      </c>
       <c r="F9" t="inlineStr">
         <is>
           <t>oui</t>
@@ -5453,7 +5669,11 @@
           <t>Outer Left Wing Pylon</t>
         </is>
       </c>
-      <c r="E10" s="7" t="n"/>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>Pylône d'aile ext. gauche</t>
+        </is>
+      </c>
       <c r="F10" t="inlineStr">
         <is>
           <t>oui</t>
@@ -5508,7 +5728,11 @@
           <t>Outer Right Wing Pylon</t>
         </is>
       </c>
-      <c r="E11" s="7" t="n"/>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>Pylône d'aile ext. droit</t>
+        </is>
+      </c>
       <c r="F11" t="inlineStr">
         <is>
           <t>oui</t>
@@ -5563,7 +5787,11 @@
           <t>Internal Guns</t>
         </is>
       </c>
-      <c r="E12" s="7" t="n"/>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>Canons internes</t>
+        </is>
+      </c>
       <c r="F12" t="inlineStr">
         <is>
           <t>oui</t>
@@ -5618,7 +5846,11 @@
           <t>Centreline Pylon</t>
         </is>
       </c>
-      <c r="E13" s="7" t="n"/>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>Pylône axial</t>
+        </is>
+      </c>
       <c r="F13" t="inlineStr">
         <is>
           <t>oui</t>
@@ -5673,7 +5905,11 @@
           <t>Inner Left Pylon</t>
         </is>
       </c>
-      <c r="E14" s="7" t="n"/>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>Pylône intérieur gauche</t>
+        </is>
+      </c>
       <c r="F14" t="inlineStr">
         <is>
           <t>oui</t>
@@ -5728,7 +5964,11 @@
           <t>Inner Right Pylon</t>
         </is>
       </c>
-      <c r="E15" s="7" t="n"/>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>Pylône intérieur droit</t>
+        </is>
+      </c>
       <c r="F15" t="inlineStr">
         <is>
           <t>oui</t>
@@ -5783,7 +6023,11 @@
           <t>Outer Left Pylon</t>
         </is>
       </c>
-      <c r="E16" s="7" t="n"/>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>Pylône extérieur gauche</t>
+        </is>
+      </c>
       <c r="F16" t="inlineStr">
         <is>
           <t>oui</t>
@@ -5838,7 +6082,11 @@
           <t>Outer Right Pylon</t>
         </is>
       </c>
-      <c r="E17" s="7" t="n"/>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>Pylône extérieur droit</t>
+        </is>
+      </c>
       <c r="F17" t="inlineStr">
         <is>
           <t>oui</t>
@@ -5893,7 +6141,11 @@
           <t>Wingtip Pylons</t>
         </is>
       </c>
-      <c r="E18" s="7" t="n"/>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>Saumons d'aile</t>
+        </is>
+      </c>
       <c r="F18" t="inlineStr">
         <is>
           <t>oui</t>
@@ -5948,7 +6200,11 @@
           <t>Inner Left Pylon</t>
         </is>
       </c>
-      <c r="E19" s="7" t="n"/>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>Pylône intérieur gauche</t>
+        </is>
+      </c>
       <c r="F19" t="inlineStr">
         <is>
           <t>oui</t>
@@ -6003,7 +6259,11 @@
           <t>Inner Right Pylon</t>
         </is>
       </c>
-      <c r="E20" s="7" t="n"/>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>Pylône intérieur droit</t>
+        </is>
+      </c>
       <c r="F20" t="inlineStr">
         <is>
           <t>oui</t>
@@ -6058,7 +6318,11 @@
           <t>Outer Left Pylon</t>
         </is>
       </c>
-      <c r="E21" s="7" t="n"/>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>Pylône extérieur gauche</t>
+        </is>
+      </c>
       <c r="F21" t="inlineStr">
         <is>
           <t>oui</t>
@@ -6113,7 +6377,11 @@
           <t>Outer Right Pylon</t>
         </is>
       </c>
-      <c r="E22" s="7" t="n"/>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>Pylône extérieur droit</t>
+        </is>
+      </c>
       <c r="F22" t="inlineStr">
         <is>
           <t>oui</t>
@@ -6168,7 +6436,11 @@
           <t>Left Internal Bay</t>
         </is>
       </c>
-      <c r="E23" s="7" t="n"/>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>Soute interne gauche</t>
+        </is>
+      </c>
       <c r="F23" t="inlineStr">
         <is>
           <t>oui</t>
@@ -6223,7 +6495,11 @@
           <t>Right Internal Bay</t>
         </is>
       </c>
-      <c r="E24" s="7" t="n"/>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>Soute interne droite</t>
+        </is>
+      </c>
       <c r="F24" t="inlineStr">
         <is>
           <t>oui</t>
@@ -6283,7 +6559,11 @@
           <t>Gun Mount</t>
         </is>
       </c>
-      <c r="E25" s="7" t="n"/>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>Support de canon</t>
+        </is>
+      </c>
       <c r="F25" t="inlineStr">
         <is>
           <t>oui</t>
@@ -6335,7 +6615,11 @@
           <t>Weapon Bay</t>
         </is>
       </c>
-      <c r="E26" s="7" t="n"/>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>Soute d'armement</t>
+        </is>
+      </c>
       <c r="F26" t="inlineStr">
         <is>
           <t>oui</t>
@@ -6390,7 +6674,11 @@
           <t>Inner Wing Pylons</t>
         </is>
       </c>
-      <c r="E27" s="7" t="n"/>
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>Pylônes d'aile intérieurs</t>
+        </is>
+      </c>
       <c r="F27" t="inlineStr">
         <is>
           <t>oui</t>
@@ -6445,7 +6733,11 @@
           <t>Middle Wing Pylons</t>
         </is>
       </c>
-      <c r="E28" s="7" t="n"/>
+      <c r="E28" s="7" t="inlineStr">
+        <is>
+          <t>Pylônes d'aile médians</t>
+        </is>
+      </c>
       <c r="F28" t="inlineStr">
         <is>
           <t>oui</t>
@@ -6500,7 +6792,11 @@
           <t>Outer Wing Pylons</t>
         </is>
       </c>
-      <c r="E29" s="7" t="n"/>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>Pylônes d'aile extérieurs</t>
+        </is>
+      </c>
       <c r="F29" t="inlineStr">
         <is>
           <t>oui</t>
@@ -6555,7 +6851,11 @@
           <t>Tail Hook</t>
         </is>
       </c>
-      <c r="E30" s="7" t="n"/>
+      <c r="E30" s="7" t="inlineStr">
+        <is>
+          <t>Crochet d'appontage</t>
+        </is>
+      </c>
       <c r="F30" s="8" t="inlineStr">
         <is>
           <t>non (sans arme)</t>
@@ -6601,7 +6901,11 @@
           <t>Center Pylon</t>
         </is>
       </c>
-      <c r="E31" s="7" t="n"/>
+      <c r="E31" s="7" t="inlineStr">
+        <is>
+          <t>Pylône central</t>
+        </is>
+      </c>
       <c r="F31" t="inlineStr">
         <is>
           <t>oui</t>
@@ -6661,7 +6965,11 @@
           <t>Left Fuselage Pylon</t>
         </is>
       </c>
-      <c r="E32" s="7" t="n"/>
+      <c r="E32" s="7" t="inlineStr">
+        <is>
+          <t>Pylône de fuselage gauche</t>
+        </is>
+      </c>
       <c r="F32" t="inlineStr">
         <is>
           <t>oui</t>
@@ -6721,7 +7029,11 @@
           <t>Right Fuselage Pylon</t>
         </is>
       </c>
-      <c r="E33" s="7" t="n"/>
+      <c r="E33" s="7" t="inlineStr">
+        <is>
+          <t>Pylône de fuselage droit</t>
+        </is>
+      </c>
       <c r="F33" t="inlineStr">
         <is>
           <t>oui</t>
@@ -6781,7 +7093,11 @@
           <t>Inner wing pylons</t>
         </is>
       </c>
-      <c r="E34" s="7" t="n"/>
+      <c r="E34" s="7" t="inlineStr">
+        <is>
+          <t>Pylônes d'aile intérieurs</t>
+        </is>
+      </c>
       <c r="F34" t="inlineStr">
         <is>
           <t>oui</t>
@@ -6836,7 +7152,11 @@
           <t>Outer wing pylons</t>
         </is>
       </c>
-      <c r="E35" s="7" t="n"/>
+      <c r="E35" s="7" t="inlineStr">
+        <is>
+          <t>Pylônes d'aile extérieurs</t>
+        </is>
+      </c>
       <c r="F35" t="inlineStr">
         <is>
           <t>oui</t>
@@ -6891,7 +7211,11 @@
           <t>Wingtip Pylons</t>
         </is>
       </c>
-      <c r="E36" s="7" t="n"/>
+      <c r="E36" s="7" t="inlineStr">
+        <is>
+          <t>Saumons d'aile</t>
+        </is>
+      </c>
       <c r="F36" t="inlineStr">
         <is>
           <t>oui</t>
@@ -6946,7 +7270,11 @@
           <t>Left Fuselage Pylon</t>
         </is>
       </c>
-      <c r="E37" s="7" t="n"/>
+      <c r="E37" s="7" t="inlineStr">
+        <is>
+          <t>Pylône de fuselage gauche</t>
+        </is>
+      </c>
       <c r="F37" t="inlineStr">
         <is>
           <t>oui</t>
@@ -7001,7 +7329,11 @@
           <t>Right Fuselage Pylon</t>
         </is>
       </c>
-      <c r="E38" s="7" t="n"/>
+      <c r="E38" s="7" t="inlineStr">
+        <is>
+          <t>Pylône de fuselage droit</t>
+        </is>
+      </c>
       <c r="F38" t="inlineStr">
         <is>
           <t>oui</t>
@@ -7056,7 +7388,11 @@
           <t>Door guns</t>
         </is>
       </c>
-      <c r="E39" s="7" t="n"/>
+      <c r="E39" s="7" t="inlineStr">
+        <is>
+          <t>Mitrailleuses de porte</t>
+        </is>
+      </c>
       <c r="F39" t="inlineStr">
         <is>
           <t>oui</t>
@@ -7111,7 +7447,11 @@
           <t>Cargo Bay</t>
         </is>
       </c>
-      <c r="E40" s="7" t="n"/>
+      <c r="E40" s="7" t="inlineStr">
+        <is>
+          <t>Soute cargo</t>
+        </is>
+      </c>
       <c r="F40" t="inlineStr">
         <is>
           <t>oui</t>
@@ -7163,7 +7503,11 @@
           <t>Cargo Bay (Front)</t>
         </is>
       </c>
-      <c r="E41" s="7" t="n"/>
+      <c r="E41" s="7" t="inlineStr">
+        <is>
+          <t>Soute cargo (avant)</t>
+        </is>
+      </c>
       <c r="F41" t="inlineStr">
         <is>
           <t>oui</t>
@@ -7223,7 +7567,11 @@
           <t>Cargo Bay (Rear)</t>
         </is>
       </c>
-      <c r="E42" s="7" t="n"/>
+      <c r="E42" s="7" t="inlineStr">
+        <is>
+          <t>Soute cargo (arrière)</t>
+        </is>
+      </c>
       <c r="F42" t="inlineStr">
         <is>
           <t>oui</t>
@@ -7275,7 +7623,11 @@
           <t>Slingload Hook</t>
         </is>
       </c>
-      <c r="E43" s="7" t="n"/>
+      <c r="E43" s="7" t="inlineStr">
+        <is>
+          <t>Crochet d'élingue</t>
+        </is>
+      </c>
       <c r="F43" t="inlineStr">
         <is>
           <t>oui</t>
@@ -7322,7 +7674,11 @@
           <t>Chin Turret</t>
         </is>
       </c>
-      <c r="E44" s="7" t="n"/>
+      <c r="E44" s="7" t="inlineStr">
+        <is>
+          <t>Tourelle de nez</t>
+        </is>
+      </c>
       <c r="F44" t="inlineStr">
         <is>
           <t>oui</t>
@@ -7377,7 +7733,11 @@
           <t>Internal Bays</t>
         </is>
       </c>
-      <c r="E45" s="7" t="n"/>
+      <c r="E45" s="7" t="inlineStr">
+        <is>
+          <t>Soutes internes</t>
+        </is>
+      </c>
       <c r="F45" t="inlineStr">
         <is>
           <t>oui</t>
@@ -7432,7 +7792,11 @@
           <t>Stub Pylons</t>
         </is>
       </c>
-      <c r="E46" s="7" t="n"/>
+      <c r="E46" s="7" t="inlineStr">
+        <is>
+          <t>Pylônes d'ailette</t>
+        </is>
+      </c>
       <c r="F46" t="inlineStr">
         <is>
           <t>oui</t>
@@ -7487,7 +7851,11 @@
           <t>Left Stub Tip Pylon</t>
         </is>
       </c>
-      <c r="E47" s="7" t="n"/>
+      <c r="E47" s="7" t="inlineStr">
+        <is>
+          <t>Pylône d'extrémité gauche</t>
+        </is>
+      </c>
       <c r="F47" t="inlineStr">
         <is>
           <t>oui</t>
@@ -7542,7 +7910,11 @@
           <t>Right Stub Tip Pylon</t>
         </is>
       </c>
-      <c r="E48" s="7" t="n"/>
+      <c r="E48" s="7" t="inlineStr">
+        <is>
+          <t>Pylône d'extrémité droit</t>
+        </is>
+      </c>
       <c r="F48" t="inlineStr">
         <is>
           <t>oui</t>
@@ -7597,7 +7969,11 @@
           <t>Internal Guns</t>
         </is>
       </c>
-      <c r="E49" s="7" t="n"/>
+      <c r="E49" s="7" t="inlineStr">
+        <is>
+          <t>Canons internes</t>
+        </is>
+      </c>
       <c r="F49" t="inlineStr">
         <is>
           <t>oui</t>
@@ -7652,7 +8028,11 @@
           <t>Weapon Bay</t>
         </is>
       </c>
-      <c r="E50" s="7" t="n"/>
+      <c r="E50" s="7" t="inlineStr">
+        <is>
+          <t>Soute d'armement</t>
+        </is>
+      </c>
       <c r="F50" t="inlineStr">
         <is>
           <t>oui</t>
@@ -7712,7 +8092,11 @@
           <t>Inner Wing Pylons</t>
         </is>
       </c>
-      <c r="E51" s="7" t="n"/>
+      <c r="E51" s="7" t="inlineStr">
+        <is>
+          <t>Pylônes d'aile intérieurs</t>
+        </is>
+      </c>
       <c r="F51" t="inlineStr">
         <is>
           <t>oui</t>
@@ -7767,7 +8151,11 @@
           <t>Outer Wing Pylons</t>
         </is>
       </c>
-      <c r="E52" s="7" t="n"/>
+      <c r="E52" s="7" t="inlineStr">
+        <is>
+          <t>Pylônes d'aile extérieurs</t>
+        </is>
+      </c>
       <c r="F52" t="inlineStr">
         <is>
           <t>oui</t>
@@ -7822,7 +8210,11 @@
           <t>Centreline Pylon</t>
         </is>
       </c>
-      <c r="E53" s="7" t="n"/>
+      <c r="E53" s="7" t="inlineStr">
+        <is>
+          <t>Pylône axial</t>
+        </is>
+      </c>
       <c r="F53" t="inlineStr">
         <is>
           <t>oui</t>
@@ -7882,7 +8274,11 @@
           <t>Tail Hook</t>
         </is>
       </c>
-      <c r="E54" s="7" t="n"/>
+      <c r="E54" s="7" t="inlineStr">
+        <is>
+          <t>Crochet d'appontage</t>
+        </is>
+      </c>
       <c r="F54" s="8" t="inlineStr">
         <is>
           <t>non (sans arme)</t>
@@ -7928,7 +8324,11 @@
           <t>Internal 35mm Autocannons</t>
         </is>
       </c>
-      <c r="E55" s="7" t="n"/>
+      <c r="E55" s="7" t="inlineStr">
+        <is>
+          <t>Canons internes de 35 mm</t>
+        </is>
+      </c>
       <c r="F55" t="inlineStr">
         <is>
           <t>oui</t>
@@ -7983,7 +8383,11 @@
           <t>Center Pylon</t>
         </is>
       </c>
-      <c r="E56" s="7" t="n"/>
+      <c r="E56" s="7" t="inlineStr">
+        <is>
+          <t>Pylône central</t>
+        </is>
+      </c>
       <c r="F56" t="inlineStr">
         <is>
           <t>oui</t>
@@ -8043,7 +8447,11 @@
           <t>Inner Fuselage Pylons</t>
         </is>
       </c>
-      <c r="E57" s="7" t="n"/>
+      <c r="E57" s="7" t="inlineStr">
+        <is>
+          <t>Pylônes de fuselage int.</t>
+        </is>
+      </c>
       <c r="F57" t="inlineStr">
         <is>
           <t>oui</t>
@@ -8103,7 +8511,11 @@
           <t>Outer Fuselage Pylons</t>
         </is>
       </c>
-      <c r="E58" s="7" t="n"/>
+      <c r="E58" s="7" t="inlineStr">
+        <is>
+          <t>Pylônes de fuselage ext.</t>
+        </is>
+      </c>
       <c r="F58" t="inlineStr">
         <is>
           <t>oui</t>
@@ -8158,7 +8570,11 @@
           <t>Inner Wing Pylons</t>
         </is>
       </c>
-      <c r="E59" s="7" t="n"/>
+      <c r="E59" s="7" t="inlineStr">
+        <is>
+          <t>Pylônes d'aile intérieurs</t>
+        </is>
+      </c>
       <c r="F59" t="inlineStr">
         <is>
           <t>oui</t>
@@ -8213,7 +8629,11 @@
           <t>Middle Wing Pylons</t>
         </is>
       </c>
-      <c r="E60" s="7" t="n"/>
+      <c r="E60" s="7" t="inlineStr">
+        <is>
+          <t>Pylônes d'aile médians</t>
+        </is>
+      </c>
       <c r="F60" t="inlineStr">
         <is>
           <t>oui</t>
@@ -8268,7 +8688,11 @@
           <t>Outer Left Wing Pylon</t>
         </is>
       </c>
-      <c r="E61" s="7" t="n"/>
+      <c r="E61" s="7" t="inlineStr">
+        <is>
+          <t>Pylône d'aile ext. gauche</t>
+        </is>
+      </c>
       <c r="F61" t="inlineStr">
         <is>
           <t>oui</t>
@@ -8323,7 +8747,11 @@
           <t>Outer Right Wing Pylon</t>
         </is>
       </c>
-      <c r="E62" s="7" t="n"/>
+      <c r="E62" s="7" t="inlineStr">
+        <is>
+          <t>Pylône d'aile ext. droit</t>
+        </is>
+      </c>
       <c r="F62" t="inlineStr">
         <is>
           <t>oui</t>
@@ -8378,7 +8806,11 @@
           <t>Cargo Bay</t>
         </is>
       </c>
-      <c r="E63" s="7" t="n"/>
+      <c r="E63" s="7" t="inlineStr">
+        <is>
+          <t>Soute cargo</t>
+        </is>
+      </c>
       <c r="F63" t="inlineStr">
         <is>
           <t>oui</t>
@@ -8438,7 +8870,11 @@
           <t>Cargo Bay (Front)</t>
         </is>
       </c>
-      <c r="E64" s="7" t="n"/>
+      <c r="E64" s="7" t="inlineStr">
+        <is>
+          <t>Soute cargo (avant)</t>
+        </is>
+      </c>
       <c r="F64" t="inlineStr">
         <is>
           <t>oui</t>
@@ -8498,7 +8934,11 @@
           <t>Cargo Bay(Rear)</t>
         </is>
       </c>
-      <c r="E65" s="7" t="n"/>
+      <c r="E65" s="7" t="inlineStr">
+        <is>
+          <t>Soute cargo (arrière)</t>
+        </is>
+      </c>
       <c r="F65" t="inlineStr">
         <is>
           <t>oui</t>
@@ -8558,7 +8998,11 @@
           <t>Floor Turret Mount</t>
         </is>
       </c>
-      <c r="E66" s="7" t="n"/>
+      <c r="E66" s="7" t="inlineStr">
+        <is>
+          <t>Tourelle ventrale</t>
+        </is>
+      </c>
       <c r="F66" t="inlineStr">
         <is>
           <t>oui</t>
@@ -8613,7 +9057,11 @@
           <t>Left Sponson Pylon</t>
         </is>
       </c>
-      <c r="E67" s="7" t="n"/>
+      <c r="E67" s="7" t="inlineStr">
+        <is>
+          <t>Pylône de flanc gauche</t>
+        </is>
+      </c>
       <c r="F67" t="inlineStr">
         <is>
           <t>oui</t>
@@ -8668,7 +9116,11 @@
           <t>Right Sponson Pylon</t>
         </is>
       </c>
-      <c r="E68" s="7" t="n"/>
+      <c r="E68" s="7" t="inlineStr">
+        <is>
+          <t>Pylône de flanc droit</t>
+        </is>
+      </c>
       <c r="F68" t="inlineStr">
         <is>
           <t>oui</t>
@@ -8723,7 +9175,11 @@
           <t>Slingload Hook</t>
         </is>
       </c>
-      <c r="E69" s="7" t="n"/>
+      <c r="E69" s="7" t="inlineStr">
+        <is>
+          <t>Crochet d'élingue</t>
+        </is>
+      </c>
       <c r="F69" t="inlineStr">
         <is>
           <t>oui</t>
@@ -8770,7 +9226,11 @@
           <t>Internal Cannon</t>
         </is>
       </c>
-      <c r="E70" s="7" t="n"/>
+      <c r="E70" s="7" t="inlineStr">
+        <is>
+          <t>Canon interne</t>
+        </is>
+      </c>
       <c r="F70" t="inlineStr">
         <is>
           <t>oui</t>
@@ -8825,7 +9285,11 @@
           <t>Centreline Pylon</t>
         </is>
       </c>
-      <c r="E71" s="7" t="n"/>
+      <c r="E71" s="7" t="inlineStr">
+        <is>
+          <t>Pylône axial</t>
+        </is>
+      </c>
       <c r="F71" t="inlineStr">
         <is>
           <t>oui</t>
@@ -8880,7 +9344,11 @@
           <t>Inner Wing Pylons</t>
         </is>
       </c>
-      <c r="E72" s="7" t="n"/>
+      <c r="E72" s="7" t="inlineStr">
+        <is>
+          <t>Pylônes d'aile intérieurs</t>
+        </is>
+      </c>
       <c r="F72" t="inlineStr">
         <is>
           <t>oui</t>
@@ -8935,7 +9403,11 @@
           <t>Mid Wing Pylons</t>
         </is>
       </c>
-      <c r="E73" s="7" t="n"/>
+      <c r="E73" s="7" t="inlineStr">
+        <is>
+          <t>Pylônes d'aile médians</t>
+        </is>
+      </c>
       <c r="F73" t="inlineStr">
         <is>
           <t>oui</t>
@@ -8990,7 +9462,11 @@
           <t>Outer Wing Pylons</t>
         </is>
       </c>
-      <c r="E74" s="7" t="n"/>
+      <c r="E74" s="7" t="inlineStr">
+        <is>
+          <t>Pylônes d'aile extérieurs</t>
+        </is>
+      </c>
       <c r="F74" t="inlineStr">
         <is>
           <t>oui</t>
@@ -9045,7 +9521,11 @@
           <t>Wingtip Pylons</t>
         </is>
       </c>
-      <c r="E75" s="7" t="n"/>
+      <c r="E75" s="7" t="inlineStr">
+        <is>
+          <t>Saumons d'aile</t>
+        </is>
+      </c>
       <c r="F75" t="inlineStr">
         <is>
           <t>oui</t>
@@ -9100,7 +9580,11 @@
           <t>Tail Hook</t>
         </is>
       </c>
-      <c r="E76" s="7" t="n"/>
+      <c r="E76" s="7" t="inlineStr">
+        <is>
+          <t>Crochet d'appontage</t>
+        </is>
+      </c>
       <c r="F76" s="8" t="inlineStr">
         <is>
           <t>non (sans arme)</t>
@@ -9146,7 +9630,11 @@
           <t>TGP</t>
         </is>
       </c>
-      <c r="E77" s="7" t="n"/>
+      <c r="E77" s="7" t="inlineStr">
+        <is>
+          <t>Nacelle de désignation</t>
+        </is>
+      </c>
       <c r="F77" t="inlineStr">
         <is>
           <t>oui</t>
@@ -9201,7 +9689,11 @@
           <t>Internal Cannon</t>
         </is>
       </c>
-      <c r="E78" s="7" t="n"/>
+      <c r="E78" s="7" t="inlineStr">
+        <is>
+          <t>Canon interne</t>
+        </is>
+      </c>
       <c r="F78" t="inlineStr">
         <is>
           <t>oui</t>
@@ -9248,7 +9740,11 @@
           <t>CenterLine Pylon</t>
         </is>
       </c>
-      <c r="E79" s="7" t="n"/>
+      <c r="E79" s="7" t="inlineStr">
+        <is>
+          <t>Pylône axial</t>
+        </is>
+      </c>
       <c r="F79" t="inlineStr">
         <is>
           <t>oui</t>
@@ -9303,7 +9799,11 @@
           <t>Inner Wing Pylons</t>
         </is>
       </c>
-      <c r="E80" s="7" t="n"/>
+      <c r="E80" s="7" t="inlineStr">
+        <is>
+          <t>Pylônes d'aile intérieurs</t>
+        </is>
+      </c>
       <c r="F80" t="inlineStr">
         <is>
           <t>oui</t>
@@ -9358,7 +9858,11 @@
           <t>Middle Wing Pylons</t>
         </is>
       </c>
-      <c r="E81" s="7" t="n"/>
+      <c r="E81" s="7" t="inlineStr">
+        <is>
+          <t>Pylônes d'aile médians</t>
+        </is>
+      </c>
       <c r="F81" t="inlineStr">
         <is>
           <t>oui</t>
@@ -9413,7 +9917,11 @@
           <t>Outer Wing Pylons</t>
         </is>
       </c>
-      <c r="E82" s="7" t="n"/>
+      <c r="E82" s="7" t="inlineStr">
+        <is>
+          <t>Pylônes d'aile extérieurs</t>
+        </is>
+      </c>
       <c r="F82" t="inlineStr">
         <is>
           <t>oui</t>
@@ -9468,7 +9976,11 @@
           <t>Wingtip</t>
         </is>
       </c>
-      <c r="E83" s="7" t="n"/>
+      <c r="E83" s="7" t="inlineStr">
+        <is>
+          <t>Saumons d'aile</t>
+        </is>
+      </c>
       <c r="F83" t="inlineStr">
         <is>
           <t>oui</t>
@@ -9523,7 +10035,11 @@
           <t>Internal Cannon</t>
         </is>
       </c>
-      <c r="E84" s="7" t="n"/>
+      <c r="E84" s="7" t="inlineStr">
+        <is>
+          <t>Canon interne</t>
+        </is>
+      </c>
       <c r="F84" t="inlineStr">
         <is>
           <t>oui</t>
@@ -9578,7 +10094,11 @@
           <t>Internal Weapon Bays</t>
         </is>
       </c>
-      <c r="E85" s="7" t="n"/>
+      <c r="E85" s="7" t="inlineStr">
+        <is>
+          <t>Soutes internes</t>
+        </is>
+      </c>
       <c r="F85" t="inlineStr">
         <is>
           <t>oui</t>
@@ -9633,7 +10153,11 @@
           <t>Wing Pylons</t>
         </is>
       </c>
-      <c r="E86" s="7" t="n"/>
+      <c r="E86" s="7" t="inlineStr">
+        <is>
+          <t>Pylônes d'aile</t>
+        </is>
+      </c>
       <c r="F86" t="inlineStr">
         <is>
           <t>oui</t>
@@ -9688,7 +10212,11 @@
           <t>Wingtip Pylons</t>
         </is>
       </c>
-      <c r="E87" s="7" t="n"/>
+      <c r="E87" s="7" t="inlineStr">
+        <is>
+          <t>Saumons d'aile</t>
+        </is>
+      </c>
       <c r="F87" t="inlineStr">
         <is>
           <t>oui</t>
@@ -9743,7 +10271,11 @@
           <t>Internal Cannon</t>
         </is>
       </c>
-      <c r="E88" s="7" t="n"/>
+      <c r="E88" s="7" t="inlineStr">
+        <is>
+          <t>Canon interne</t>
+        </is>
+      </c>
       <c r="F88" t="inlineStr">
         <is>
           <t>oui</t>
@@ -9798,7 +10330,11 @@
           <t>Weapon Bays (inner)</t>
         </is>
       </c>
-      <c r="E89" s="7" t="n"/>
+      <c r="E89" s="7" t="inlineStr">
+        <is>
+          <t>Soutes (intérieures)</t>
+        </is>
+      </c>
       <c r="F89" t="inlineStr">
         <is>
           <t>oui</t>
@@ -9853,7 +10389,11 @@
           <t>Weapon Bays (outer)</t>
         </is>
       </c>
-      <c r="E90" s="7" t="n"/>
+      <c r="E90" s="7" t="inlineStr">
+        <is>
+          <t>Soutes (extérieures)</t>
+        </is>
+      </c>
       <c r="F90" t="inlineStr">
         <is>
           <t>oui</t>
@@ -9908,7 +10448,11 @@
           <t>Inner wing pylons</t>
         </is>
       </c>
-      <c r="E91" s="7" t="n"/>
+      <c r="E91" s="7" t="inlineStr">
+        <is>
+          <t>Pylônes d'aile intérieurs</t>
+        </is>
+      </c>
       <c r="F91" t="inlineStr">
         <is>
           <t>oui</t>
@@ -9963,7 +10507,11 @@
           <t>Outer wing pylons</t>
         </is>
       </c>
-      <c r="E92" s="7" t="n"/>
+      <c r="E92" s="7" t="inlineStr">
+        <is>
+          <t>Pylônes d'aile extérieurs</t>
+        </is>
+      </c>
       <c r="F92" t="inlineStr">
         <is>
           <t>oui</t>
@@ -10018,7 +10566,11 @@
           <t>Left Weapon Bay</t>
         </is>
       </c>
-      <c r="E93" s="7" t="n"/>
+      <c r="E93" s="7" t="inlineStr">
+        <is>
+          <t>Soute gauche</t>
+        </is>
+      </c>
       <c r="F93" t="inlineStr">
         <is>
           <t>oui</t>
@@ -10073,7 +10625,11 @@
           <t>Right Weapon Bay</t>
         </is>
       </c>
-      <c r="E94" s="7" t="n"/>
+      <c r="E94" s="7" t="inlineStr">
+        <is>
+          <t>Soute droite</t>
+        </is>
+      </c>
       <c r="F94" t="inlineStr">
         <is>
           <t>oui</t>
@@ -10128,7 +10684,11 @@
           <t>JammingPod1</t>
         </is>
       </c>
-      <c r="E95" s="7" t="n"/>
+      <c r="E95" s="7" t="inlineStr">
+        <is>
+          <t>Nacelle de brouillage</t>
+        </is>
+      </c>
       <c r="F95" t="inlineStr">
         <is>
           <t>oui</t>
@@ -10183,7 +10743,11 @@
           <t>Internal Cannon</t>
         </is>
       </c>
-      <c r="E96" s="7" t="n"/>
+      <c r="E96" s="7" t="inlineStr">
+        <is>
+          <t>Canon interne</t>
+        </is>
+      </c>
       <c r="F96" t="inlineStr">
         <is>
           <t>oui</t>
@@ -10238,7 +10802,11 @@
           <t>Forward Weapon Bay</t>
         </is>
       </c>
-      <c r="E97" s="7" t="n"/>
+      <c r="E97" s="7" t="inlineStr">
+        <is>
+          <t>Soute avant</t>
+        </is>
+      </c>
       <c r="F97" t="inlineStr">
         <is>
           <t>oui</t>
@@ -10293,7 +10861,11 @@
           <t>Rear Weapon Bay</t>
         </is>
       </c>
-      <c r="E98" s="7" t="n"/>
+      <c r="E98" s="7" t="inlineStr">
+        <is>
+          <t>Soute arrière</t>
+        </is>
+      </c>
       <c r="F98" t="inlineStr">
         <is>
           <t>oui</t>
@@ -10348,7 +10920,11 @@
           <t>Side Weapon Bays</t>
         </is>
       </c>
-      <c r="E99" s="7" t="n"/>
+      <c r="E99" s="7" t="inlineStr">
+        <is>
+          <t>Soutes latérales</t>
+        </is>
+      </c>
       <c r="F99" t="inlineStr">
         <is>
           <t>oui</t>
@@ -10403,7 +10979,11 @@
           <t>Inner Wing Pylons</t>
         </is>
       </c>
-      <c r="E100" s="7" t="n"/>
+      <c r="E100" s="7" t="inlineStr">
+        <is>
+          <t>Pylônes d'aile intérieurs</t>
+        </is>
+      </c>
       <c r="F100" t="inlineStr">
         <is>
           <t>oui</t>
@@ -10458,7 +11038,11 @@
           <t>Outer Wing Pylons</t>
         </is>
       </c>
-      <c r="E101" s="7" t="n"/>
+      <c r="E101" s="7" t="inlineStr">
+        <is>
+          <t>Pylônes d'aile extérieurs</t>
+        </is>
+      </c>
       <c r="F101" t="inlineStr">
         <is>
           <t>oui</t>
@@ -10513,7 +11097,11 @@
           <t>Tail Hook</t>
         </is>
       </c>
-      <c r="E102" s="7" t="n"/>
+      <c r="E102" s="7" t="inlineStr">
+        <is>
+          <t>Crochet d'appontage</t>
+        </is>
+      </c>
       <c r="F102" s="8" t="inlineStr">
         <is>
           <t>non (sans arme)</t>
@@ -10559,7 +11147,11 @@
           <t>Internal Cannon</t>
         </is>
       </c>
-      <c r="E103" s="7" t="n"/>
+      <c r="E103" s="7" t="inlineStr">
+        <is>
+          <t>Canon interne</t>
+        </is>
+      </c>
       <c r="F103" t="inlineStr">
         <is>
           <t>oui</t>
@@ -10614,7 +11206,11 @@
           <t>Combined Weapon Bay</t>
         </is>
       </c>
-      <c r="E104" s="7" t="n"/>
+      <c r="E104" s="7" t="inlineStr">
+        <is>
+          <t>Soute combinée</t>
+        </is>
+      </c>
       <c r="F104" t="inlineStr">
         <is>
           <t>oui</t>
@@ -10674,7 +11270,11 @@
           <t>Forward Weapon Bay</t>
         </is>
       </c>
-      <c r="E105" s="7" t="n"/>
+      <c r="E105" s="7" t="inlineStr">
+        <is>
+          <t>Soute avant</t>
+        </is>
+      </c>
       <c r="F105" t="inlineStr">
         <is>
           <t>oui</t>
@@ -10729,7 +11329,11 @@
           <t>Rear Weapon Bay</t>
         </is>
       </c>
-      <c r="E106" s="7" t="n"/>
+      <c r="E106" s="7" t="inlineStr">
+        <is>
+          <t>Soute arrière</t>
+        </is>
+      </c>
       <c r="F106" t="inlineStr">
         <is>
           <t>oui</t>
@@ -10784,7 +11388,11 @@
           <t>Front Fuselage Pylons</t>
         </is>
       </c>
-      <c r="E107" s="7" t="n"/>
+      <c r="E107" s="7" t="inlineStr">
+        <is>
+          <t>Pylônes de fuselage avant</t>
+        </is>
+      </c>
       <c r="F107" t="inlineStr">
         <is>
           <t>oui</t>
@@ -10839,7 +11447,11 @@
           <t>Rear Fuselage Pylons</t>
         </is>
       </c>
-      <c r="E108" s="7" t="n"/>
+      <c r="E108" s="7" t="inlineStr">
+        <is>
+          <t>Pylônes de fuselage arrière</t>
+        </is>
+      </c>
       <c r="F108" t="inlineStr">
         <is>
           <t>oui</t>
@@ -10894,7 +11506,11 @@
           <t>Inner Wing Pylons</t>
         </is>
       </c>
-      <c r="E109" s="7" t="n"/>
+      <c r="E109" s="7" t="inlineStr">
+        <is>
+          <t>Pylônes d'aile intérieurs</t>
+        </is>
+      </c>
       <c r="F109" t="inlineStr">
         <is>
           <t>oui</t>
@@ -10949,7 +11565,11 @@
           <t>Middle Wing Pylons</t>
         </is>
       </c>
-      <c r="E110" s="7" t="n"/>
+      <c r="E110" s="7" t="inlineStr">
+        <is>
+          <t>Pylônes d'aile médians</t>
+        </is>
+      </c>
       <c r="F110" t="inlineStr">
         <is>
           <t>oui</t>
@@ -11004,7 +11624,11 @@
           <t>Outer Wing Pylons</t>
         </is>
       </c>
-      <c r="E111" s="7" t="n"/>
+      <c r="E111" s="7" t="inlineStr">
+        <is>
+          <t>Pylônes d'aile extérieurs</t>
+        </is>
+      </c>
       <c r="F111" t="inlineStr">
         <is>
           <t>oui</t>
@@ -11059,7 +11683,11 @@
           <t>Internal Laser Mount</t>
         </is>
       </c>
-      <c r="E112" s="7" t="n"/>
+      <c r="E112" s="7" t="inlineStr">
+        <is>
+          <t>Laser interne</t>
+        </is>
+      </c>
       <c r="F112" t="inlineStr">
         <is>
           <t>oui</t>
@@ -11114,7 +11742,11 @@
           <t>Weapon Bay</t>
         </is>
       </c>
-      <c r="E113" s="7" t="n"/>
+      <c r="E113" s="7" t="inlineStr">
+        <is>
+          <t>Soute d'armement</t>
+        </is>
+      </c>
       <c r="F113" t="inlineStr">
         <is>
           <t>oui</t>
@@ -11169,7 +11801,11 @@
           <t>Dorsal Mount</t>
         </is>
       </c>
-      <c r="E114" s="7" t="n"/>
+      <c r="E114" s="7" t="inlineStr">
+        <is>
+          <t>Support dorsal</t>
+        </is>
+      </c>
       <c r="F114" t="inlineStr">
         <is>
           <t>oui</t>
@@ -11224,7 +11860,11 @@
           <t>Inner Wing Pylons</t>
         </is>
       </c>
-      <c r="E115" s="7" t="n"/>
+      <c r="E115" s="7" t="inlineStr">
+        <is>
+          <t>Pylônes d'aile intérieurs</t>
+        </is>
+      </c>
       <c r="F115" t="inlineStr">
         <is>
           <t>oui</t>
@@ -11279,7 +11919,11 @@
           <t>Outer Wing Pylons</t>
         </is>
       </c>
-      <c r="E116" s="7" t="n"/>
+      <c r="E116" s="7" t="inlineStr">
+        <is>
+          <t>Pylônes d'aile extérieurs</t>
+        </is>
+      </c>
       <c r="F116" t="inlineStr">
         <is>
           <t>oui</t>
@@ -11334,7 +11978,11 @@
           <t>Wing Pylons</t>
         </is>
       </c>
-      <c r="E117" s="7" t="n"/>
+      <c r="E117" s="7" t="inlineStr">
+        <is>
+          <t>Pylônes d'aile</t>
+        </is>
+      </c>
       <c r="F117" t="inlineStr">
         <is>
           <t>oui</t>
@@ -11389,7 +12037,11 @@
           <t>Cargo Bay Rear</t>
         </is>
       </c>
-      <c r="E118" s="7" t="n"/>
+      <c r="E118" s="7" t="inlineStr">
+        <is>
+          <t>Soute cargo (arrière)</t>
+        </is>
+      </c>
       <c r="F118" t="inlineStr">
         <is>
           <t>oui</t>
@@ -11441,7 +12093,11 @@
           <t>Cargo Bay Front</t>
         </is>
       </c>
-      <c r="E119" s="7" t="n"/>
+      <c r="E119" s="7" t="inlineStr">
+        <is>
+          <t>Soute cargo (avant)</t>
+        </is>
+      </c>
       <c r="F119" t="inlineStr">
         <is>
           <t>oui</t>
@@ -11493,7 +12149,11 @@
           <t>Mission Bay</t>
         </is>
       </c>
-      <c r="E120" s="7" t="n"/>
+      <c r="E120" s="7" t="inlineStr">
+        <is>
+          <t>Soute de mission</t>
+        </is>
+      </c>
       <c r="F120" t="inlineStr">
         <is>
           <t>oui</t>
@@ -11545,7 +12205,11 @@
           <t>Bomb Bay (2x)</t>
         </is>
       </c>
-      <c r="E121" s="7" t="n"/>
+      <c r="E121" s="7" t="inlineStr">
+        <is>
+          <t>Soute à bombes (×2)</t>
+        </is>
+      </c>
       <c r="F121" t="inlineStr">
         <is>
           <t>oui</t>
@@ -11605,7 +12269,11 @@
           <t>Radome</t>
         </is>
       </c>
-      <c r="E122" s="7" t="n"/>
+      <c r="E122" s="7" t="inlineStr">
+        <is>
+          <t>Radôme</t>
+        </is>
+      </c>
       <c r="F122" t="inlineStr">
         <is>
           <t>oui</t>
@@ -11665,7 +12333,11 @@
           <t>Front Turret</t>
         </is>
       </c>
-      <c r="E123" s="7" t="n"/>
+      <c r="E123" s="7" t="inlineStr">
+        <is>
+          <t>Tourelle avant</t>
+        </is>
+      </c>
       <c r="F123" t="inlineStr">
         <is>
           <t>oui</t>
@@ -11725,7 +12397,11 @@
           <t>Rear Turret</t>
         </is>
       </c>
-      <c r="E124" s="7" t="n"/>
+      <c r="E124" s="7" t="inlineStr">
+        <is>
+          <t>Tourelle arrière</t>
+        </is>
+      </c>
       <c r="F124" t="inlineStr">
         <is>
           <t>oui</t>
@@ -11785,7 +12461,11 @@
           <t>-</t>
         </is>
       </c>
-      <c r="E125" s="7" t="n"/>
+      <c r="E125" s="7" t="inlineStr">
+        <is>
+          <t>Crochet d'appontage</t>
+        </is>
+      </c>
       <c r="F125" s="8" t="inlineStr">
         <is>
           <t>non (sans arme)</t>
@@ -11831,7 +12511,11 @@
           <t>Internal Gun</t>
         </is>
       </c>
-      <c r="E126" s="7" t="n"/>
+      <c r="E126" s="7" t="inlineStr">
+        <is>
+          <t>Canon interne</t>
+        </is>
+      </c>
       <c r="F126" t="inlineStr">
         <is>
           <t>oui</t>
@@ -11886,7 +12570,11 @@
           <t>Heater Bays</t>
         </is>
       </c>
-      <c r="E127" s="7" t="n"/>
+      <c r="E127" s="7" t="inlineStr">
+        <is>
+          <t>Soutes à missiles IR</t>
+        </is>
+      </c>
       <c r="F127" t="inlineStr">
         <is>
           <t>oui</t>
@@ -11941,7 +12629,11 @@
           <t>Left Bay</t>
         </is>
       </c>
-      <c r="E128" s="7" t="n"/>
+      <c r="E128" s="7" t="inlineStr">
+        <is>
+          <t>Soute gauche</t>
+        </is>
+      </c>
       <c r="F128" t="inlineStr">
         <is>
           <t>oui</t>
@@ -12001,7 +12693,11 @@
           <t>Right Bay</t>
         </is>
       </c>
-      <c r="E129" s="7" t="n"/>
+      <c r="E129" s="7" t="inlineStr">
+        <is>
+          <t>Soute droite</t>
+        </is>
+      </c>
       <c r="F129" t="inlineStr">
         <is>
           <t>oui</t>
@@ -12061,7 +12757,11 @@
           <t>Outer L Bay</t>
         </is>
       </c>
-      <c r="E130" s="7" t="n"/>
+      <c r="E130" s="7" t="inlineStr">
+        <is>
+          <t>Soute extérieure gauche</t>
+        </is>
+      </c>
       <c r="F130" t="inlineStr">
         <is>
           <t>oui</t>
@@ -12121,7 +12821,11 @@
           <t>Outer R Bay</t>
         </is>
       </c>
-      <c r="E131" s="7" t="n"/>
+      <c r="E131" s="7" t="inlineStr">
+        <is>
+          <t>Soute extérieure droite</t>
+        </is>
+      </c>
       <c r="F131" t="inlineStr">
         <is>
           <t>oui</t>
@@ -12181,7 +12885,11 @@
           <t>Inner L Bay</t>
         </is>
       </c>
-      <c r="E132" s="7" t="n"/>
+      <c r="E132" s="7" t="inlineStr">
+        <is>
+          <t>Soute intérieure gauche</t>
+        </is>
+      </c>
       <c r="F132" t="inlineStr">
         <is>
           <t>oui</t>
@@ -12241,7 +12949,11 @@
           <t>Inner R Bay</t>
         </is>
       </c>
-      <c r="E133" s="7" t="n"/>
+      <c r="E133" s="7" t="inlineStr">
+        <is>
+          <t>Soute intérieure droite</t>
+        </is>
+      </c>
       <c r="F133" t="inlineStr">
         <is>
           <t>oui</t>
@@ -12301,7 +13013,11 @@
           <t>Inner Wing Pylons</t>
         </is>
       </c>
-      <c r="E134" s="7" t="n"/>
+      <c r="E134" s="7" t="inlineStr">
+        <is>
+          <t>Pylônes d'aile intérieurs</t>
+        </is>
+      </c>
       <c r="F134" t="inlineStr">
         <is>
           <t>oui</t>
@@ -12356,7 +13072,11 @@
           <t>Outer Wing Pylons</t>
         </is>
       </c>
-      <c r="E135" s="7" t="n"/>
+      <c r="E135" s="7" t="inlineStr">
+        <is>
+          <t>Pylônes d'aile extérieurs</t>
+        </is>
+      </c>
       <c r="F135" t="inlineStr">
         <is>
           <t>oui</t>
@@ -12411,7 +13131,11 @@
           <t>Tailhook</t>
         </is>
       </c>
-      <c r="E136" s="7" t="n"/>
+      <c r="E136" s="7" t="inlineStr">
+        <is>
+          <t>Crochet d'appontage</t>
+        </is>
+      </c>
       <c r="F136" s="8" t="inlineStr">
         <is>
           <t>non (sans arme)</t>
@@ -12457,7 +13181,11 @@
           <t>Inner Weapon Bays (Combined)</t>
         </is>
       </c>
-      <c r="E137" s="7" t="n"/>
+      <c r="E137" s="7" t="inlineStr">
+        <is>
+          <t>Soutes int. (combinées)</t>
+        </is>
+      </c>
       <c r="F137" t="inlineStr">
         <is>
           <t>oui</t>
@@ -12517,7 +13245,11 @@
           <t>Inner Weapon Bays (Rear)</t>
         </is>
       </c>
-      <c r="E138" s="7" t="n"/>
+      <c r="E138" s="7" t="inlineStr">
+        <is>
+          <t>Soutes int. (arrière)</t>
+        </is>
+      </c>
       <c r="F138" t="inlineStr">
         <is>
           <t>oui</t>
@@ -12577,7 +13309,11 @@
           <t>Inner Weapon Bays (Front)</t>
         </is>
       </c>
-      <c r="E139" s="7" t="n"/>
+      <c r="E139" s="7" t="inlineStr">
+        <is>
+          <t>Soutes int. (avant)</t>
+        </is>
+      </c>
       <c r="F139" t="inlineStr">
         <is>
           <t>oui</t>
@@ -12637,7 +13373,11 @@
           <t>Outer weapon bays</t>
         </is>
       </c>
-      <c r="E140" s="7" t="n"/>
+      <c r="E140" s="7" t="inlineStr">
+        <is>
+          <t>Soutes extérieures</t>
+        </is>
+      </c>
       <c r="F140" t="inlineStr">
         <is>
           <t>oui</t>
@@ -12692,7 +13432,11 @@
           <t>Internal Cannon</t>
         </is>
       </c>
-      <c r="E141" s="7" t="n"/>
+      <c r="E141" s="7" t="inlineStr">
+        <is>
+          <t>Canon interne</t>
+        </is>
+      </c>
       <c r="F141" t="inlineStr">
         <is>
           <t>oui</t>
@@ -12747,7 +13491,11 @@
           <t>Centreline Pylon</t>
         </is>
       </c>
-      <c r="E142" s="7" t="n"/>
+      <c r="E142" s="7" t="inlineStr">
+        <is>
+          <t>Pylône axial</t>
+        </is>
+      </c>
       <c r="F142" t="inlineStr">
         <is>
           <t>oui</t>
@@ -12807,7 +13555,11 @@
           <t>Forward Weapon Bay</t>
         </is>
       </c>
-      <c r="E143" s="7" t="n"/>
+      <c r="E143" s="7" t="inlineStr">
+        <is>
+          <t>Soute avant</t>
+        </is>
+      </c>
       <c r="F143" t="inlineStr">
         <is>
           <t>oui</t>
@@ -12867,7 +13619,11 @@
           <t>Rear Weapon Bay</t>
         </is>
       </c>
-      <c r="E144" s="7" t="n"/>
+      <c r="E144" s="7" t="inlineStr">
+        <is>
+          <t>Soute arrière</t>
+        </is>
+      </c>
       <c r="F144" t="inlineStr">
         <is>
           <t>oui</t>
@@ -12927,7 +13683,11 @@
           <t>Heater Bays</t>
         </is>
       </c>
-      <c r="E145" s="7" t="n"/>
+      <c r="E145" s="7" t="inlineStr">
+        <is>
+          <t>Soutes à missiles IR</t>
+        </is>
+      </c>
       <c r="F145" t="inlineStr">
         <is>
           <t>oui</t>
@@ -12982,7 +13742,11 @@
           <t>Wing Glove Pylons</t>
         </is>
       </c>
-      <c r="E146" s="7" t="n"/>
+      <c r="E146" s="7" t="inlineStr">
+        <is>
+          <t>Pylônes d'emplanture</t>
+        </is>
+      </c>
       <c r="F146" t="inlineStr">
         <is>
           <t>oui</t>
@@ -13037,7 +13801,11 @@
           <t>Wing Pylons</t>
         </is>
       </c>
-      <c r="E147" s="7" t="n"/>
+      <c r="E147" s="7" t="inlineStr">
+        <is>
+          <t>Pylônes d'aile</t>
+        </is>
+      </c>
       <c r="F147" t="inlineStr">
         <is>
           <t>oui</t>
@@ -13092,7 +13860,11 @@
           <t>Tail Hook</t>
         </is>
       </c>
-      <c r="E148" s="7" t="n"/>
+      <c r="E148" s="7" t="inlineStr">
+        <is>
+          <t>Crochet d'appontage</t>
+        </is>
+      </c>
       <c r="F148" s="8" t="inlineStr">
         <is>
           <t>non (sans arme)</t>
@@ -13138,7 +13910,11 @@
           <t>Forward Weapon Bay</t>
         </is>
       </c>
-      <c r="E149" s="7" t="n"/>
+      <c r="E149" s="7" t="inlineStr">
+        <is>
+          <t>Soute avant</t>
+        </is>
+      </c>
       <c r="F149" t="inlineStr">
         <is>
           <t>oui</t>
@@ -13198,7 +13974,11 @@
           <t>Rear Weapon Bay</t>
         </is>
       </c>
-      <c r="E150" s="7" t="n"/>
+      <c r="E150" s="7" t="inlineStr">
+        <is>
+          <t>Soute arrière</t>
+        </is>
+      </c>
       <c r="F150" t="inlineStr">
         <is>
           <t>oui</t>
@@ -13258,7 +14038,11 @@
           <t>Combined Weapon Bays</t>
         </is>
       </c>
-      <c r="E151" s="7" t="n"/>
+      <c r="E151" s="7" t="inlineStr">
+        <is>
+          <t>Soutes combinées</t>
+        </is>
+      </c>
       <c r="F151" t="inlineStr">
         <is>
           <t>oui</t>
@@ -13318,7 +14102,11 @@
           <t>Wing Pylons</t>
         </is>
       </c>
-      <c r="E152" s="7" t="n"/>
+      <c r="E152" s="7" t="inlineStr">
+        <is>
+          <t>Pylônes d'aile</t>
+        </is>
+      </c>
       <c r="F152" t="inlineStr">
         <is>
           <t>oui</t>
@@ -13373,7 +14161,11 @@
           <t>Heater Bays</t>
         </is>
       </c>
-      <c r="E153" s="7" t="n"/>
+      <c r="E153" s="7" t="inlineStr">
+        <is>
+          <t>Soutes à missiles IR</t>
+        </is>
+      </c>
       <c r="F153" t="inlineStr">
         <is>
           <t>oui</t>

</xml_diff>

<commit_message>
Wiki avions : V5, maquette de la fiche appareil (vraies données, 3 thèmes, cotes 7.3) et captures
Repli des canons fixes lu en jeu (emplacements internes à canon).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ta6XHrP5piK3ygC9quASBg
</commit_message>
<xml_diff>
--- a/data/Avions_wiki.xlsx
+++ b/data/Avions_wiki.xlsx
@@ -1077,6 +1077,9 @@
           <t>non</t>
         </is>
       </c>
+      <c r="AI2" t="n">
+        <v>3</v>
+      </c>
       <c r="AJ2" t="n">
         <v>24</v>
       </c>
@@ -1130,6 +1133,11 @@
           <t>MiG-15s in the big '85 :wilt: :sob:</t>
         </is>
       </c>
+      <c r="BC2" t="inlineStr">
+        <is>
+          <t>Canons fixes = 3 (emplacements internes à canon, lus en jeu).</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1246,6 +1254,9 @@
           <t>non</t>
         </is>
       </c>
+      <c r="AI3" t="n">
+        <v>2</v>
+      </c>
       <c r="AJ3" t="n">
         <v>48</v>
       </c>
@@ -1302,6 +1313,11 @@
           <t>Designed for counter insurgency operations and low-intensity battlefields, the CI-22 Cricket features robust landing gear and short takeoff and landing capability, allowing it to operate from unprepared fields. While lacking in speed and survivability, the CI-22 possesses remarkable agility and the ability to mount an array of weapon types</t>
         </is>
       </c>
+      <c r="BC3" t="inlineStr">
+        <is>
+          <t>Canons fixes = 2 (emplacements internes à canon, lus en jeu).</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1409,6 +1425,9 @@
           <t>non</t>
         </is>
       </c>
+      <c r="AI4" t="n">
+        <v>2</v>
+      </c>
       <c r="AJ4" t="n">
         <v>48</v>
       </c>
@@ -1467,7 +1486,7 @@
       </c>
       <c r="BC4" t="inlineStr">
         <is>
-          <t>Masse à vide non renseignée dans la fiche du jeu Masse à vide inconnue : N/A (A15 : somme des pièces concordante pour 12/21 appareils seulement, moins de 80 %).</t>
+          <t>Masse à vide non renseignée dans la fiche du jeu Canons fixes = 2 (emplacements internes à canon, lus en jeu). Masse à vide inconnue : N/A (A15 : somme des pièces concordante pour 12/21 appareils seulement, moins de 80 %).</t>
         </is>
       </c>
     </row>
@@ -1568,6 +1587,9 @@
           <t>non</t>
         </is>
       </c>
+      <c r="AI5" t="n">
+        <v>0</v>
+      </c>
       <c r="AJ5" t="n">
         <v>72</v>
       </c>
@@ -1745,6 +1767,9 @@
           <t>oui</t>
         </is>
       </c>
+      <c r="AI6" t="n">
+        <v>0</v>
+      </c>
       <c r="AJ6" t="n">
         <v>64</v>
       </c>
@@ -1920,6 +1945,9 @@
           <t>oui</t>
         </is>
       </c>
+      <c r="AI7" t="n">
+        <v>0</v>
+      </c>
       <c r="AJ7" t="n">
         <v>64</v>
       </c>
@@ -2083,6 +2111,9 @@
           <t>non</t>
         </is>
       </c>
+      <c r="AI8" t="n">
+        <v>0</v>
+      </c>
       <c r="AJ8" t="n">
         <v>64</v>
       </c>
@@ -2424,6 +2455,9 @@
           <t>oui</t>
         </is>
       </c>
+      <c r="AI10" t="n">
+        <v>2</v>
+      </c>
       <c r="AJ10" t="n">
         <v>50</v>
       </c>
@@ -2480,6 +2514,11 @@
           <t>Although an older design, this light supersonic fighter is exceptionally agile and highly suited to air superiority missions with options for limited low-level ground attack. Twin engines provide an incredible TWR and top speed whilst a centreline internal weapon bay reduces payload drag.</t>
         </is>
       </c>
+      <c r="BC10" t="inlineStr">
+        <is>
+          <t>Canons fixes = 2 (emplacements internes à canon, lus en jeu).</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2762,6 +2801,9 @@
           <t>non</t>
         </is>
       </c>
+      <c r="AI12" t="n">
+        <v>0</v>
+      </c>
       <c r="AJ12" t="n">
         <v>144</v>
       </c>
@@ -2930,6 +2972,9 @@
           <t>oui</t>
         </is>
       </c>
+      <c r="AI13" t="n">
+        <v>1</v>
+      </c>
       <c r="AJ13" t="n">
         <v>64</v>
       </c>
@@ -2988,7 +3033,7 @@
       </c>
       <c r="BC13" t="inlineStr">
         <is>
-          <t>Vitesse max. = valeur déclarée par le mod (très supérieure au jeu de base)</t>
+          <t>Vitesse max. = valeur déclarée par le mod (très supérieure au jeu de base) Canons fixes = 1 (emplacements internes à canon, lus en jeu).</t>
         </is>
       </c>
     </row>
@@ -3110,6 +3155,9 @@
           <t>oui</t>
         </is>
       </c>
+      <c r="AI14" t="n">
+        <v>1</v>
+      </c>
       <c r="AJ14" t="n">
         <v>64</v>
       </c>
@@ -3168,7 +3216,7 @@
       </c>
       <c r="BC14" t="inlineStr">
         <is>
-          <t>Embarque aussi une arme événementielle (3S-RMM, ex-MMR-S3 montée à l'envers)</t>
+          <t>Embarque aussi une arme événementielle (3S-RMM, ex-MMR-S3 montée à l'envers) Canons fixes = 1 (emplacements internes à canon, lus en jeu).</t>
         </is>
       </c>
     </row>
@@ -3290,6 +3338,9 @@
           <t>oui</t>
         </is>
       </c>
+      <c r="AI15" t="n">
+        <v>1</v>
+      </c>
       <c r="AJ15" t="n">
         <v>64</v>
       </c>
@@ -3346,6 +3397,11 @@
           <t>The FS-12 Revoker is built for agility above all else, capable of extreme maneuvers at almost any speed. Internal weapon bays help reduce drag, allowing supersonic speeds even at low altitudes and with heavy payloads. While less stealthy than newer fighters, the Revoker remains a cost-effective means of establishing air superiority.</t>
         </is>
       </c>
+      <c r="BC15" t="inlineStr">
+        <is>
+          <t>Canons fixes = 1 (emplacements internes à canon, lus en jeu).</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3465,6 +3521,9 @@
           <t>oui</t>
         </is>
       </c>
+      <c r="AI16" t="n">
+        <v>1</v>
+      </c>
       <c r="AJ16" t="n">
         <v>72</v>
       </c>
@@ -3521,6 +3580,11 @@
           <t>A compact and advanced multirole fighter, the Vortex is capable of operating vertically from small carriers and remaining undetected thanks to outstanding stealth characteristics. While fast, agile, and stealthy when lightly loaded, these characteristics can suffer when carrying a heavy payload of weapons.</t>
         </is>
       </c>
+      <c r="BC16" t="inlineStr">
+        <is>
+          <t>Canons fixes = 1 (emplacements internes à canon, lus en jeu).</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3637,6 +3701,9 @@
           <t>non</t>
         </is>
       </c>
+      <c r="AI17" t="n">
+        <v>0</v>
+      </c>
       <c r="AJ17" t="n">
         <v>32</v>
       </c>
@@ -3820,6 +3887,9 @@
           <t>oui</t>
         </is>
       </c>
+      <c r="AI18" t="n">
+        <v>1</v>
+      </c>
       <c r="AJ18" t="n">
         <v>72</v>
       </c>
@@ -3876,6 +3946,11 @@
           <t>A large, carrier capable, twin engine multirole fighter, the Ifrit is equally suited to air superiority and ground attack missions. It features excellent thrust and maneuverability alongside reduced radar signature and powerful sensors. Two internal weapon bays plus two additional side bays for heat-seeking missiles allow the Ifrit to carry a significant internal payload without impacting stealth or top speed.</t>
         </is>
       </c>
+      <c r="BC18" t="inlineStr">
+        <is>
+          <t>Canons fixes = 1 (emplacements internes à canon, lus en jeu).</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3995,6 +4070,9 @@
           <t>oui</t>
         </is>
       </c>
+      <c r="AI19" t="n">
+        <v>1</v>
+      </c>
       <c r="AJ19" t="n">
         <v>96</v>
       </c>
@@ -4053,7 +4131,7 @@
       </c>
       <c r="BC19" t="inlineStr">
         <is>
-          <t>Vitesse max. = valeur déclarée par le mod (très supérieure au jeu de base)</t>
+          <t>Vitesse max. = valeur déclarée par le mod (très supérieure au jeu de base) Canons fixes = 1 (emplacements internes à canon, lus en jeu).</t>
         </is>
       </c>
     </row>
@@ -4175,6 +4253,9 @@
           <t>oui</t>
         </is>
       </c>
+      <c r="AI20" t="n">
+        <v>0</v>
+      </c>
       <c r="AJ20" t="n">
         <v>86</v>
       </c>
@@ -4347,6 +4428,9 @@
           <t>oui</t>
         </is>
       </c>
+      <c r="AI21" t="n">
+        <v>0</v>
+      </c>
       <c r="AJ21" t="n">
         <v>256</v>
       </c>
@@ -4513,6 +4597,9 @@
           <t>oui</t>
         </is>
       </c>
+      <c r="AI22" t="n">
+        <v>1</v>
+      </c>
       <c r="AJ22" t="n">
         <v>72</v>
       </c>
@@ -4571,7 +4658,7 @@
       </c>
       <c r="BC22" t="inlineStr">
         <is>
-          <t>Masse à vide non renseignée dans la fiche du jeu ; Vitesse max. = valeur déclarée par le mod (très supérieure au jeu de base) Masse à vide inconnue : N/A (A15 : somme des pièces concordante pour 12/21 appareils seulement, moins de 80 %).</t>
+          <t>Masse à vide non renseignée dans la fiche du jeu ; Vitesse max. = valeur déclarée par le mod (très supérieure au jeu de base) Canons fixes = 1 (emplacements internes à canon, lus en jeu). Masse à vide inconnue : N/A (A15 : somme des pièces concordante pour 12/21 appareils seulement, moins de 80 %).</t>
         </is>
       </c>
     </row>
@@ -4693,6 +4780,9 @@
           <t>oui</t>
         </is>
       </c>
+      <c r="AI23" t="n">
+        <v>0</v>
+      </c>
       <c r="AJ23" t="n">
         <v>86</v>
       </c>
@@ -4865,6 +4955,9 @@
           <t>oui</t>
         </is>
       </c>
+      <c r="AI24" t="n">
+        <v>1</v>
+      </c>
       <c r="AJ24" t="n">
         <v>84</v>
       </c>
@@ -4923,7 +5016,7 @@
       </c>
       <c r="BC24" t="inlineStr">
         <is>
-          <t>Vitesse max. = valeur déclarée par le mod (très supérieure au jeu de base)</t>
+          <t>Vitesse max. = valeur déclarée par le mod (très supérieure au jeu de base) Canons fixes = 1 (emplacements internes à canon, lus en jeu).</t>
         </is>
       </c>
     </row>
@@ -5044,6 +5137,9 @@
         <is>
           <t>oui</t>
         </is>
+      </c>
+      <c r="AI25" t="n">
+        <v>0</v>
       </c>
       <c r="AJ25" t="n">
         <v>90</v>

</xml_diff>

<commit_message>
Wiki avions : amendement v3.6, charge utile = masse d'armement maximale des emplacements (tous les appareils)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ta6XHrP5piK3ygC9quASBg
</commit_message>
<xml_diff>
--- a/data/Avions_wiki.xlsx
+++ b/data/Avions_wiki.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A24"/>
+  <dimension ref="A1:A25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -611,15 +611,22 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t xml:space="preserve">  • Charge utile (v3.6) : masse d'armement maximale sur l'ensemble des emplacements (points × arme la plus lourde, cargo exclu), meilleure combinaison d'emplacements compatibles. Pour un appareil cargo, force la valeur dans Corrections (« Charge utile (kg) »).</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
           <t xml:space="preserve">  • Masse à vide manquante (A15) : somme des pièces du prefab seulement si elle concorde à ±15 % pour au moins 80 % des appareils ; sinon N/A (voir la colonne Notes).</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" t="inlineStr"/>
-    </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
         <is>
           <t>Mise à jour : remplace data/sources/NO-stats.xlsx si besoin, modifie les colonnes jaunes ou Corrections, enregistre, ferme Excel, puis double-clique sur mettre_a_jour.bat : le classeur et aircraft.json sont régénérés et copiés à côté de la DLL du mod.</t>
         </is>
@@ -1025,7 +1032,7 @@
         <v>6.1</v>
       </c>
       <c r="M2" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="N2" t="n">
         <v>1</v>
@@ -1058,7 +1065,7 @@
         <v>6106</v>
       </c>
       <c r="X2" t="n">
-        <v>2506</v>
+        <v>584</v>
       </c>
       <c r="Y2" t="n">
         <v>1100</v>
@@ -1203,7 +1210,7 @@
         <v>2.2</v>
       </c>
       <c r="M3" t="n">
-        <v>1</v>
+        <v>3.7</v>
       </c>
       <c r="N3" t="n">
         <v>1.4</v>
@@ -1236,7 +1243,7 @@
         <v>4800</v>
       </c>
       <c r="X3" t="n">
-        <v>950</v>
+        <v>2510</v>
       </c>
       <c r="Y3" t="n">
         <v>500</v>
@@ -1383,6 +1390,9 @@
       <c r="L4" t="n">
         <v>3</v>
       </c>
+      <c r="M4" t="n">
+        <v>1.8</v>
+      </c>
       <c r="N4" t="n">
         <v>1.8</v>
       </c>
@@ -1409,6 +1419,9 @@
       </c>
       <c r="W4" t="n">
         <v>6000</v>
+      </c>
+      <c r="X4" t="n">
+        <v>2188</v>
       </c>
       <c r="Y4" t="n">
         <v>1050</v>
@@ -1555,6 +1568,9 @@
       <c r="L5" t="n">
         <v>1.4</v>
       </c>
+      <c r="M5" t="n">
+        <v>1.4</v>
+      </c>
       <c r="N5" t="n">
         <v>2.2</v>
       </c>
@@ -1578,6 +1594,9 @@
       </c>
       <c r="W5" t="n">
         <v>8500</v>
+      </c>
+      <c r="X5" t="n">
+        <v>1624</v>
       </c>
       <c r="Y5" t="n">
         <v>1000</v>
@@ -1719,7 +1738,7 @@
         <v>5.3</v>
       </c>
       <c r="M6" t="n">
-        <v>4.2</v>
+        <v>4.5</v>
       </c>
       <c r="N6" t="n">
         <v>2.6</v>
@@ -1752,7 +1771,7 @@
         <v>10800</v>
       </c>
       <c r="X6" t="n">
-        <v>5600</v>
+        <v>3840</v>
       </c>
       <c r="Y6" t="n">
         <v>2071.4</v>
@@ -1895,7 +1914,7 @@
         <v>5.3</v>
       </c>
       <c r="M7" t="n">
-        <v>2.8</v>
+        <v>3.3</v>
       </c>
       <c r="N7" t="n">
         <v>3</v>
@@ -1928,7 +1947,7 @@
         <v>10050</v>
       </c>
       <c r="X7" t="n">
-        <v>4850</v>
+        <v>2494</v>
       </c>
       <c r="Y7" t="n">
         <v>3650.3</v>
@@ -2074,7 +2093,7 @@
         <v>1.8</v>
       </c>
       <c r="M8" t="n">
-        <v>6</v>
+        <v>2.2</v>
       </c>
       <c r="N8" t="n">
         <v>3.3</v>
@@ -2104,7 +2123,7 @@
         <v>15500</v>
       </c>
       <c r="X8" t="n">
-        <v>8240</v>
+        <v>2350</v>
       </c>
       <c r="Y8" t="n">
         <v>1400</v>
@@ -2241,7 +2260,7 @@
         <v>1</v>
       </c>
       <c r="M9" t="n">
-        <v>1.9</v>
+        <v>4.1</v>
       </c>
       <c r="N9" t="n">
         <v>3.7</v>
@@ -2271,7 +2290,7 @@
         <v>10500</v>
       </c>
       <c r="X9" t="n">
-        <v>3240</v>
+        <v>3036</v>
       </c>
       <c r="Y9" t="n">
         <v>1050</v>
@@ -2408,7 +2427,7 @@
         <v>8.4</v>
       </c>
       <c r="M10" t="n">
-        <v>2.4</v>
+        <v>3</v>
       </c>
       <c r="N10" t="n">
         <v>4.1</v>
@@ -2441,7 +2460,7 @@
         <v>10000</v>
       </c>
       <c r="X10" t="n">
-        <v>4000</v>
+        <v>2434</v>
       </c>
       <c r="Y10" t="n">
         <v>1400</v>
@@ -2592,7 +2611,7 @@
         <v>3.3</v>
       </c>
       <c r="M11" t="n">
-        <v>6.9</v>
+        <v>8</v>
       </c>
       <c r="N11" t="n">
         <v>4.5</v>
@@ -2625,7 +2644,7 @@
         <v>19000</v>
       </c>
       <c r="X11" t="n">
-        <v>13800</v>
+        <v>9300</v>
       </c>
       <c r="Y11" t="n">
         <v>4800</v>
@@ -2768,7 +2787,7 @@
         <v>2.6</v>
       </c>
       <c r="M12" t="n">
-        <v>9.6</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="N12" t="n">
         <v>6.5</v>
@@ -2798,7 +2817,7 @@
         <v>53500</v>
       </c>
       <c r="X12" t="n">
-        <v>46240</v>
+        <v>21126</v>
       </c>
       <c r="Y12" t="n">
         <v>8600</v>
@@ -2928,7 +2947,7 @@
         <v>9.6</v>
       </c>
       <c r="M13" t="n">
-        <v>5.1</v>
+        <v>5.7</v>
       </c>
       <c r="N13" t="n">
         <v>4.9</v>
@@ -2961,7 +2980,7 @@
         <v>16240</v>
       </c>
       <c r="X13" t="n">
-        <v>7740</v>
+        <v>6079</v>
       </c>
       <c r="Y13" t="n">
         <v>3320</v>
@@ -3112,7 +3131,7 @@
         <v>7.7</v>
       </c>
       <c r="M14" t="n">
-        <v>5.5</v>
+        <v>5.3</v>
       </c>
       <c r="N14" t="n">
         <v>5.3</v>
@@ -3145,7 +3164,7 @@
         <v>16500</v>
       </c>
       <c r="X14" t="n">
-        <v>7920</v>
+        <v>4530</v>
       </c>
       <c r="Y14" t="n">
         <v>3300</v>
@@ -3296,7 +3315,7 @@
         <v>6.5</v>
       </c>
       <c r="M15" t="n">
-        <v>3.7</v>
+        <v>4.9</v>
       </c>
       <c r="N15" t="n">
         <v>5.7</v>
@@ -3329,7 +3348,7 @@
         <v>16000</v>
       </c>
       <c r="X15" t="n">
-        <v>5300</v>
+        <v>4240</v>
       </c>
       <c r="Y15" t="n">
         <v>3200</v>
@@ -3480,7 +3499,7 @@
         <v>6.9</v>
       </c>
       <c r="M16" t="n">
-        <v>3.7</v>
+        <v>6.1</v>
       </c>
       <c r="N16" t="n">
         <v>6.1</v>
@@ -3513,7 +3532,7 @@
         <v>16000</v>
       </c>
       <c r="X16" t="n">
-        <v>5300</v>
+        <v>6220</v>
       </c>
       <c r="Y16" t="n">
         <v>2800</v>
@@ -3664,7 +3683,7 @@
         <v>5.7</v>
       </c>
       <c r="M17" t="n">
-        <v>6.4</v>
+        <v>2.6</v>
       </c>
       <c r="N17" t="n">
         <v>6.9</v>
@@ -3697,7 +3716,7 @@
         <v>23814</v>
       </c>
       <c r="X17" t="n">
-        <v>10434</v>
+        <v>2420</v>
       </c>
       <c r="Y17" t="n">
         <v>8250</v>
@@ -3848,7 +3867,7 @@
         <v>7.3</v>
       </c>
       <c r="M18" t="n">
-        <v>7.8</v>
+        <v>6.9</v>
       </c>
       <c r="N18" t="n">
         <v>7.3</v>
@@ -3881,7 +3900,7 @@
         <v>30000</v>
       </c>
       <c r="X18" t="n">
-        <v>19300</v>
+        <v>8398</v>
       </c>
       <c r="Y18" t="n">
         <v>8200</v>
@@ -4032,7 +4051,7 @@
         <v>8.800000000000001</v>
       </c>
       <c r="M19" t="n">
-        <v>8.199999999999999</v>
+        <v>8.4</v>
       </c>
       <c r="N19" t="n">
         <v>7.7</v>
@@ -4065,7 +4084,7 @@
         <v>39800</v>
       </c>
       <c r="X19" t="n">
-        <v>20700</v>
+        <v>13700</v>
       </c>
       <c r="Y19" t="n">
         <v>12000</v>
@@ -4216,7 +4235,7 @@
         <v>4.5</v>
       </c>
       <c r="M20" t="n">
-        <v>4.6</v>
+        <v>7.3</v>
       </c>
       <c r="N20" t="n">
         <v>8</v>
@@ -4249,7 +4268,7 @@
         <v>26000</v>
       </c>
       <c r="X20" t="n">
-        <v>6960</v>
+        <v>8670</v>
       </c>
       <c r="Y20" t="n">
         <v>5500</v>
@@ -4392,7 +4411,7 @@
         <v>3.7</v>
       </c>
       <c r="M21" t="n">
-        <v>10</v>
+        <v>9.6</v>
       </c>
       <c r="N21" t="n">
         <v>8.4</v>
@@ -4425,7 +4444,7 @@
         <v>130000</v>
       </c>
       <c r="X21" t="n">
-        <v>85000</v>
+        <v>28500</v>
       </c>
       <c r="Y21" t="n">
         <v>26500</v>
@@ -4570,6 +4589,9 @@
       <c r="L22" t="n">
         <v>9.199999999999999</v>
       </c>
+      <c r="M22" t="n">
+        <v>7.7</v>
+      </c>
       <c r="N22" t="n">
         <v>8.800000000000001</v>
       </c>
@@ -4596,6 +4618,9 @@
       </c>
       <c r="W22" t="n">
         <v>38000</v>
+      </c>
+      <c r="X22" t="n">
+        <v>9200</v>
       </c>
       <c r="Y22" t="n">
         <v>8200</v>
@@ -4746,7 +4771,7 @@
         <v>4.1</v>
       </c>
       <c r="M23" t="n">
-        <v>9.1</v>
+        <v>10</v>
       </c>
       <c r="N23" t="n">
         <v>9.199999999999999</v>
@@ -4779,7 +4804,7 @@
         <v>115000</v>
       </c>
       <c r="X23" t="n">
-        <v>44930</v>
+        <v>33000</v>
       </c>
       <c r="Y23" t="n">
         <v>24997.9</v>
@@ -4922,7 +4947,7 @@
         <v>10</v>
       </c>
       <c r="M24" t="n">
-        <v>7.3</v>
+        <v>6.5</v>
       </c>
       <c r="N24" t="n">
         <v>9.6</v>
@@ -4955,7 +4980,7 @@
         <v>32500</v>
       </c>
       <c r="X24" t="n">
-        <v>14000</v>
+        <v>7840</v>
       </c>
       <c r="Y24" t="n">
         <v>7950</v>
@@ -5106,7 +5131,7 @@
         <v>8</v>
       </c>
       <c r="M25" t="n">
-        <v>8.699999999999999</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="N25" t="n">
         <v>10</v>
@@ -5139,7 +5164,7 @@
         <v>62000</v>
       </c>
       <c r="X25" t="n">
-        <v>28000</v>
+        <v>22020</v>
       </c>
       <c r="Y25" t="n">
         <v>18200</v>

</xml_diff>